<commit_message>
generacion de ticket 2
</commit_message>
<xml_diff>
--- a/data/CODIGO_DE_FALLAS.xlsx
+++ b/data/CODIGO_DE_FALLAS.xlsx
@@ -1,42 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Proyectos_Personales\Sistema_Prediccion_Repuestos_Insumos\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB77CBDB-09C0-4F9E-876D-D28DBEFA2FC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-28920" yWindow="-7650" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Hoja1" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="54">
+  <si>
+    <t>CODIGO</t>
+  </si>
+  <si>
+    <t>FALLA</t>
+  </si>
+  <si>
+    <t>REFERENCIA</t>
+  </si>
   <si>
     <t>051</t>
   </si>
@@ -83,114 +67,72 @@
     <t xml:space="preserve">  Microtélefono dañado/ parlante saturado</t>
   </si>
   <si>
-    <t>117</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Deteriorado</t>
   </si>
   <si>
     <t xml:space="preserve"> accesorios, conectores, perillas, pines en mal estado </t>
   </si>
   <si>
-    <t>160</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Contacto o conexión defectuoso</t>
   </si>
   <si>
     <t xml:space="preserve"> sulfatado, corroído</t>
   </si>
   <si>
-    <t>169</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Voltaje incorrecto</t>
   </si>
   <si>
     <t xml:space="preserve"> polaridad invertida, fuera de valor nominal</t>
   </si>
   <si>
-    <t>255</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Falla de potencia de salida</t>
   </si>
   <si>
     <t xml:space="preserve"> potencia baja, Roe alto, Amplificador F/S</t>
   </si>
   <si>
-    <t>266</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Soldadura deficiente</t>
   </si>
   <si>
     <t xml:space="preserve"> encendido intermitente </t>
   </si>
   <si>
-    <t>472</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Fusible quemado</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>481</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Recalentamiento</t>
   </si>
   <si>
-    <t>585</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Cortado</t>
   </si>
   <si>
     <t xml:space="preserve"> accesorios</t>
   </si>
   <si>
-    <t>622</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Mojado o húmedo</t>
   </si>
   <si>
-    <t>694</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Video defectuoso</t>
   </si>
   <si>
     <t xml:space="preserve"> no da imagen, imagen distorsionada</t>
   </si>
   <si>
-    <t>701</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Deformado</t>
   </si>
   <si>
-    <t>750</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Faltante</t>
   </si>
   <si>
-    <t>816</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Impedancia incorrecta</t>
   </si>
   <si>
     <t xml:space="preserve"> antena cortada, Cable dañado, Acoplador F/S</t>
   </si>
   <si>
-    <t>900</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Quemado</t>
   </si>
   <si>
@@ -231,34 +173,19 @@
   </si>
   <si>
     <t xml:space="preserve"> Sistema operativo dañado, disco rígido F/S</t>
-  </si>
-  <si>
-    <t>CODIGO</t>
-  </si>
-  <si>
-    <t>FALLA</t>
-  </si>
-  <si>
-    <t>REFERENCIA</t>
-  </si>
-  <si>
-    <t>No se encuentra en la lista de fallas</t>
-  </si>
-  <si>
-    <t>Otra falla</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -311,44 +238,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -378,12 +305,12 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -422,247 +349,306 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
+                <a:tint val="100000"/>
                 <a:shade val="100000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="87.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.285714285714286" customWidth="1"/>
+    <col min="2" max="2" width="30.285714285714285" customWidth="1"/>
+    <col min="3" max="3" width="42.142857142857146" customWidth="1"/>
+    <col min="4" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>66</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>67</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>15</v>
+      <c r="A7">
+        <v>117</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>18</v>
+      <c r="A8">
+        <v>160</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>21</v>
+      <c r="A9">
+        <v>169</v>
       </c>
       <c r="B9" t="s">
         <v>22</v>
@@ -672,179 +658,170 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="A10">
+        <v>255</v>
+      </c>
+      <c r="B10" t="s">
         <v>24</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>25</v>
       </c>
-      <c r="C10" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>266</v>
+      </c>
+      <c r="B11" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="C11" t="s">
         <v>27</v>
       </c>
-      <c r="B11" t="s">
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>472</v>
+      </c>
+      <c r="B12" t="s">
         <v>28</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C12" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>481</v>
+      </c>
+      <c r="B13" t="s">
         <v>30</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C13" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>585</v>
+      </c>
+      <c r="B14" t="s">
         <v>31</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C14" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>622</v>
+      </c>
+      <c r="B15" t="s">
         <v>33</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>694</v>
+      </c>
+      <c r="B16" t="s">
         <v>34</v>
       </c>
-      <c r="C13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="C16" t="s">
         <v>35</v>
       </c>
-      <c r="B14" t="s">
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>701</v>
+      </c>
+      <c r="B17" t="s">
         <v>36</v>
       </c>
-      <c r="C14" t="s">
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>750</v>
+      </c>
+      <c r="B18" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="C18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>816</v>
+      </c>
+      <c r="B19" t="s">
         <v>38</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C19" t="s">
         <v>39</v>
       </c>
-      <c r="C15" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>900</v>
+      </c>
+      <c r="B20" t="s">
         <v>40</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C20" t="s">
         <v>41</v>
-      </c>
-      <c r="C16" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>43</v>
-      </c>
-      <c r="B17" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>45</v>
-      </c>
-      <c r="B18" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>47</v>
-      </c>
-      <c r="B19" t="s">
-        <v>48</v>
-      </c>
-      <c r="C19" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>50</v>
-      </c>
-      <c r="B20" t="s">
-        <v>51</v>
-      </c>
-      <c r="C20" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="C21" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B22" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="C22" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="B23" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="C23" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="B24" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="C24" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>0</v>
-      </c>
-      <c r="B25" t="s">
-        <v>69</v>
-      </c>
-      <c r="C25" t="s">
-        <v>68</v>
-      </c>
-    </row>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>